<commit_message>
4.0.6 state model updates
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/InputData/trans/BVS/BAU Vehicle Subsidy.xlsx
+++ b/InputData/trans/BVS/BAU Vehicle Subsidy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\state-eps-data\AL\trans\BVS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF656001-9AF3-4BA3-A6D7-75A46CEB7A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F227171-827D-4807-8C3E-E0617B2AEBDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="338" yWindow="338" windowWidth="16200" windowHeight="9307" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1557,12 +1557,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G51"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="69.3984375" customWidth="1"/>
+    <col min="2" max="2" width="69.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>30</v>
       </c>
       <c r="C1" s="37">
-        <v>46266</v>
+        <v>46274</v>
       </c>
       <c r="F1" s="35" t="s">
         <v>31</v>
@@ -1579,7 +1579,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="str">
         <f>LOOKUP(B1,F2:G51,G2:G51)</f>
         <v>AL</v>
@@ -1591,7 +1591,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>37</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>40</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F6" s="36" t="s">
         <v>43</v>
       </c>
@@ -1635,7 +1635,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7" s="59" t="s">
         <v>236</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>237</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>238</v>
       </c>
@@ -1668,7 +1668,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>239</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <v>2026</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="F12" s="36" t="s">
         <v>58</v>
@@ -1699,7 +1699,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F13" s="36" t="s">
         <v>60</v>
       </c>
@@ -1707,7 +1707,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" s="4"/>
       <c r="F14" s="36" t="s">
         <v>62</v>
@@ -1716,7 +1716,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>235</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>45</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>48</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F18" s="36" t="s">
         <v>70</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F20" s="36" t="s">
         <v>74</v>
       </c>
@@ -1776,7 +1776,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F21" s="36" t="s">
         <v>76</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F22" s="36" t="s">
         <v>78</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F23" s="36" t="s">
         <v>80</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F24" s="36" t="s">
         <v>82</v>
       </c>
@@ -1808,7 +1808,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F25" s="36" t="s">
         <v>84</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
       <c r="F26" s="36" t="s">
         <v>86</v>
@@ -1825,7 +1825,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F27" s="36" t="s">
         <v>88</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B28" s="4"/>
       <c r="F28" s="36" t="s">
         <v>90</v>
@@ -1842,7 +1842,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F29" s="36" t="s">
         <v>92</v>
       </c>
@@ -1850,7 +1850,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F30" s="36" t="s">
         <v>94</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="F31" s="36" t="s">
         <v>96</v>
@@ -1867,7 +1867,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F32" s="36" t="s">
         <v>98</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="33" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="33" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F33" s="36" t="s">
         <v>100</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="34" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F34" s="36" t="s">
         <v>102</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="35" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F35" s="36" t="s">
         <v>104</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="36" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F36" s="36" t="s">
         <v>106</v>
       </c>
@@ -1907,7 +1907,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="37" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F37" s="36" t="s">
         <v>108</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="38" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F38" s="36" t="s">
         <v>110</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="39" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F39" s="36" t="s">
         <v>112</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F40" s="36" t="s">
         <v>114</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="41" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F41" s="36" t="s">
         <v>116</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F42" s="36" t="s">
         <v>118</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="43" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F43" s="36" t="s">
         <v>120</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="44" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F44" s="36" t="s">
         <v>122</v>
       </c>
@@ -1971,7 +1971,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="45" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F45" s="36" t="s">
         <v>124</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="46" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F46" s="36" t="s">
         <v>126</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="47" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F47" s="36" t="s">
         <v>128</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="48" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F48" s="36" t="s">
         <v>130</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="49" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F49" s="36" t="s">
         <v>132</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="50" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F50" s="36" t="s">
         <v>134</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="51" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F51" s="36" t="s">
         <v>136</v>
       </c>
@@ -2039,12 +2039,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -2139,7 +2139,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -2614,7 +2614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -2815,12 +2815,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -3010,7 +3010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -3591,7 +3591,7 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3603,12 +3603,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -3703,7 +3703,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -3808,7 +3808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -4093,7 +4093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -4198,7 +4198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -4293,7 +4293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -4410,13 +4410,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
-    <col min="4" max="4" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -4511,7 +4511,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -4533,33 +4533,26 @@
         <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!E14</f>
         <v>28423.919999999998</v>
       </c>
-      <c r="G2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!F14</f>
-        <v>27596.04</v>
-      </c>
-      <c r="H2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!G14</f>
-        <v>26792.280000000002</v>
-      </c>
-      <c r="I2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!H14</f>
-        <v>26011.920000000002</v>
-      </c>
-      <c r="J2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!I14</f>
-        <v>25254.28</v>
-      </c>
-      <c r="K2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!J14</f>
-        <v>24518.719999999998</v>
-      </c>
-      <c r="L2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!K14</f>
-        <v>23804.6</v>
-      </c>
-      <c r="M2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!L14</f>
-        <v>23111.239999999998</v>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -4616,7 +4609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -4711,7 +4704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -4806,7 +4799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -4901,7 +4894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -4912,7 +4905,7 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <f t="shared" ref="D6:M6" si="0">D2</f>
+        <f t="shared" ref="D6:F6" si="0">D2</f>
         <v>30140.120000000003</v>
       </c>
       <c r="E6">
@@ -4924,32 +4917,25 @@
         <v>28423.919999999998</v>
       </c>
       <c r="G6">
-        <f t="shared" si="0"/>
-        <v>27596.04</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <f t="shared" si="0"/>
-        <v>26792.280000000002</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
-        <v>26011.920000000002</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <f t="shared" si="0"/>
-        <v>25254.28</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <f t="shared" si="0"/>
-        <v>24518.719999999998</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <f t="shared" si="0"/>
-        <v>23804.6</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <f t="shared" si="0"/>
-        <v>23111.239999999998</v>
+        <v>0</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -5006,7 +4992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -5101,7 +5087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -5112,7 +5098,7 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <f t="shared" ref="D8:M8" si="1">D2</f>
+        <f t="shared" ref="D8:F8" si="1">D2</f>
         <v>30140.120000000003</v>
       </c>
       <c r="E8">
@@ -5124,32 +5110,25 @@
         <v>28423.919999999998</v>
       </c>
       <c r="G8">
-        <f t="shared" si="1"/>
-        <v>27596.04</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <f t="shared" si="1"/>
-        <v>26792.280000000002</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <f t="shared" si="1"/>
-        <v>26011.920000000002</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <f t="shared" si="1"/>
-        <v>25254.28</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <f t="shared" si="1"/>
-        <v>24518.719999999998</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <f t="shared" si="1"/>
-        <v>23804.6</v>
+        <v>0</v>
       </c>
       <c r="M8">
-        <f t="shared" si="1"/>
-        <v>23111.239999999998</v>
+        <v>0</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -5217,12 +5196,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -5317,7 +5296,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -5412,7 +5391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -5507,7 +5486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -5602,7 +5581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -5697,7 +5676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -5792,7 +5771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -5887,7 +5866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -5993,12 +5972,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -6093,7 +6072,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -6188,7 +6167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -6283,7 +6262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -6378,7 +6357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -6473,7 +6452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -6568,7 +6547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -6663,7 +6642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -6769,12 +6748,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -6869,7 +6848,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -6964,7 +6943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -7059,7 +7038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -7154,7 +7133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -7249,7 +7228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -7344,7 +7323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -7439,7 +7418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -7545,12 +7524,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -7645,7 +7624,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -7740,7 +7719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -7835,7 +7814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -7930,7 +7909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -8025,7 +8004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -8120,7 +8099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -8215,7 +8194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -8318,34 +8297,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AO107"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.3984375" customWidth="1"/>
-    <col min="2" max="2" width="15.73046875" customWidth="1"/>
-    <col min="3" max="3" width="19.1328125" customWidth="1"/>
-    <col min="4" max="7" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.3984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="11.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>2021</v>
       </c>
@@ -8437,7 +8416,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -8532,7 +8511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
@@ -8627,7 +8606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="55" t="s">
         <v>5</v>
       </c>
@@ -8722,41 +8701,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -8768,7 +8747,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="38"/>
       <c r="B17" s="46"/>
       <c r="C17" s="38"/>
@@ -8781,7 +8760,7 @@
       <c r="J17" s="39"/>
       <c r="K17" s="38"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="38"/>
       <c r="B18" s="46"/>
       <c r="C18" s="38"/>
@@ -8797,7 +8776,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="8"/>
       <c r="B19" s="47"/>
       <c r="C19" s="8"/>
@@ -8809,7 +8788,7 @@
       <c r="I19" s="48"/>
       <c r="J19" s="48"/>
     </row>
-    <row r="20" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
       <c r="B20" s="47"/>
       <c r="C20" s="10"/>
@@ -8824,7 +8803,7 @@
       <c r="L20" s="10"/>
       <c r="M20" s="11"/>
     </row>
-    <row r="21" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="47"/>
       <c r="C21" s="8"/>
@@ -8839,7 +8818,7 @@
       <c r="L21" s="10"/>
       <c r="M21" s="11"/>
     </row>
-    <row r="22" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
       <c r="B22" s="47"/>
       <c r="C22" s="8"/>
@@ -8854,7 +8833,7 @@
       <c r="L22" s="10"/>
       <c r="M22" s="11"/>
     </row>
-    <row r="23" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="47"/>
       <c r="C23" s="8"/>
@@ -8869,7 +8848,7 @@
       <c r="L23" s="10"/>
       <c r="M23" s="11"/>
     </row>
-    <row r="24" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
       <c r="B24" s="50"/>
       <c r="C24" s="7"/>
@@ -8883,7 +8862,7 @@
       <c r="K24" s="7"/>
       <c r="R24" s="12"/>
     </row>
-    <row r="25" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
       <c r="B25" s="50"/>
       <c r="C25" s="7"/>
@@ -8896,7 +8875,7 @@
       <c r="J25" s="8"/>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
       <c r="B26" s="50"/>
       <c r="C26" s="7"/>
@@ -8908,7 +8887,7 @@
       <c r="I26" s="8"/>
       <c r="J26" s="8"/>
     </row>
-    <row r="27" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="50"/>
       <c r="C27" s="7"/>
@@ -8920,7 +8899,7 @@
       <c r="I27" s="8"/>
       <c r="J27" s="8"/>
     </row>
-    <row r="28" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="50"/>
       <c r="C28" s="7"/>
@@ -8932,7 +8911,7 @@
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
     </row>
-    <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" s="50"/>
       <c r="C29" s="7"/>
@@ -8944,7 +8923,7 @@
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
     </row>
-    <row r="30" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" s="50"/>
       <c r="C30" s="7"/>
@@ -8957,7 +8936,7 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
       <c r="B31" s="50"/>
       <c r="C31" s="7"/>
@@ -8969,7 +8948,7 @@
       <c r="I31" s="48"/>
       <c r="J31" s="48"/>
     </row>
-    <row r="32" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" s="50"/>
       <c r="C32" s="7"/>
@@ -8982,7 +8961,7 @@
       <c r="J32" s="51"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>
       <c r="B33" s="47"/>
       <c r="C33" s="8"/>
@@ -8995,15 +8974,15 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
     </row>
-    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -9015,7 +8994,7 @@
       <c r="I36" s="8"/>
       <c r="J36" s="8"/>
     </row>
-    <row r="37" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D37" s="39"/>
       <c r="E37" s="39"/>
       <c r="F37" s="39"/>
@@ -9024,7 +9003,7 @@
       <c r="I37" s="39"/>
       <c r="J37" s="39"/>
     </row>
-    <row r="38" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D38" s="39"/>
       <c r="E38" s="39"/>
       <c r="F38" s="39"/>
@@ -9033,7 +9012,7 @@
       <c r="I38" s="39"/>
       <c r="J38" s="39"/>
     </row>
-    <row r="39" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -9045,7 +9024,7 @@
       <c r="I39" s="48"/>
       <c r="J39" s="48"/>
     </row>
-    <row r="40" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="10"/>
@@ -9057,7 +9036,7 @@
       <c r="I40" s="48"/>
       <c r="J40" s="48"/>
     </row>
-    <row r="41" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -9069,7 +9048,7 @@
       <c r="I41" s="8"/>
       <c r="J41" s="8"/>
     </row>
-    <row r="42" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -9081,7 +9060,7 @@
       <c r="I42" s="8"/>
       <c r="J42" s="8"/>
     </row>
-    <row r="43" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -9093,7 +9072,7 @@
       <c r="I43" s="49"/>
       <c r="J43" s="49"/>
     </row>
-    <row r="44" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -9105,7 +9084,7 @@
       <c r="I44" s="8"/>
       <c r="J44" s="8"/>
     </row>
-    <row r="45" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
@@ -9117,7 +9096,7 @@
       <c r="I45" s="8"/>
       <c r="J45" s="8"/>
     </row>
-    <row r="46" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
@@ -9129,7 +9108,7 @@
       <c r="I46" s="8"/>
       <c r="J46" s="8"/>
     </row>
-    <row r="47" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
@@ -9141,7 +9120,7 @@
       <c r="I47" s="8"/>
       <c r="J47" s="8"/>
     </row>
-    <row r="48" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:11" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
@@ -9153,7 +9132,7 @@
       <c r="I48" s="8"/>
       <c r="J48" s="8"/>
     </row>
-    <row r="49" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
@@ -9165,7 +9144,7 @@
       <c r="I49" s="8"/>
       <c r="J49" s="8"/>
     </row>
-    <row r="50" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
@@ -9177,7 +9156,7 @@
       <c r="I50" s="8"/>
       <c r="J50" s="8"/>
     </row>
-    <row r="51" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
       <c r="B51" s="7"/>
       <c r="C51" s="7"/>
@@ -9189,7 +9168,7 @@
       <c r="I51" s="48"/>
       <c r="J51" s="48"/>
     </row>
-    <row r="52" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
@@ -9201,7 +9180,7 @@
       <c r="I52" s="51"/>
       <c r="J52" s="51"/>
     </row>
-    <row r="53" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -9213,15 +9192,15 @@
       <c r="I53" s="8"/>
       <c r="J53" s="8"/>
     </row>
-    <row r="54" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:32" s="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8"/>
       <c r="B54" s="8"/>
     </row>
-    <row r="55" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
     </row>
-    <row r="56" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -9233,24 +9212,24 @@
       <c r="I56" s="8"/>
       <c r="J56" s="7"/>
     </row>
-    <row r="57" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A57" s="13"/>
     </row>
-    <row r="58" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A58" s="5"/>
     </row>
-    <row r="59" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A59" s="5"/>
     </row>
-    <row r="60" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A60" s="5"/>
     </row>
-    <row r="61" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A61" s="55" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:32" x14ac:dyDescent="0.25">
       <c r="C62">
         <v>2021</v>
       </c>
@@ -9342,7 +9321,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="63" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>3</v>
       </c>
@@ -9467,7 +9446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>4</v>
       </c>
@@ -9592,15 +9571,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A65" s="5"/>
     </row>
-    <row r="66" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="67" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C67">
         <v>2021</v>
       </c>
@@ -9692,7 +9671,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="68" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>3</v>
       </c>
@@ -9818,7 +9797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>4</v>
       </c>
@@ -9943,7 +9922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:41" x14ac:dyDescent="0.25">
       <c r="D73" s="21" t="s">
         <v>11</v>
       </c>
@@ -9954,7 +9933,7 @@
       <c r="I73" s="21"/>
       <c r="J73" s="21"/>
     </row>
-    <row r="74" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:41" x14ac:dyDescent="0.25">
       <c r="D74" s="21" t="s">
         <v>12</v>
       </c>
@@ -9965,7 +9944,7 @@
       <c r="I74" s="21"/>
       <c r="J74" s="21"/>
     </row>
-    <row r="75" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:41" x14ac:dyDescent="0.25">
       <c r="D75" s="21">
         <v>2020</v>
       </c>
@@ -9988,7 +9967,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="76" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:41" x14ac:dyDescent="0.25">
       <c r="D76" s="40">
         <v>0.2467</v>
       </c>
@@ -10013,7 +9992,7 @@
         <v>0.46560000000000001</v>
       </c>
     </row>
-    <row r="78" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:41" x14ac:dyDescent="0.25">
       <c r="B78" s="21"/>
       <c r="C78" s="21">
         <v>2012</v>
@@ -10133,7 +10112,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="79" spans="1:41" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:41" x14ac:dyDescent="0.25">
       <c r="B79" s="21" t="s">
         <v>13</v>
       </c>
@@ -10255,7 +10234,7 @@
         <v>0.35314299999999998</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>14</v>
       </c>
@@ -10275,7 +10254,7 @@
       <c r="K82" s="16"/>
       <c r="L82" s="14"/>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>16</v>
       </c>
@@ -10298,7 +10277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>17</v>
       </c>
@@ -10321,7 +10300,7 @@
         <v>0.985564</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>18</v>
       </c>
@@ -10344,7 +10323,7 @@
         <v>0.969831</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>19</v>
       </c>
@@ -10367,7 +10346,7 @@
         <v>0.96868200000000004</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>20</v>
       </c>
@@ -10390,7 +10369,7 @@
         <v>0.95661399999999996</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>21</v>
       </c>
@@ -10413,7 +10392,7 @@
         <v>0.93666000000000005</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -10436,7 +10415,7 @@
         <v>0.914327</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>23</v>
       </c>
@@ -10459,7 +10438,7 @@
         <v>0.89805500000000005</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>24</v>
       </c>
@@ -10482,7 +10461,7 @@
         <v>0.88711099999999998</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>25</v>
       </c>
@@ -10505,7 +10484,7 @@
         <v>0.84730399999999995</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>26</v>
       </c>
@@ -10528,7 +10507,7 @@
         <v>0.78452100000000002</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>27</v>
       </c>
@@ -10545,7 +10524,7 @@
         <v>0.75350300000000003</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>28</v>
       </c>
@@ -10562,7 +10541,7 @@
         <v>0.73191600000000001</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2025</v>
       </c>
@@ -10578,7 +10557,7 @@
         <v>0.71059799999999995</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2026</v>
       </c>
@@ -10594,7 +10573,7 @@
         <v>0.68990099999999999</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2027</v>
       </c>
@@ -10610,7 +10589,7 @@
         <v>0.66980700000000004</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>2028</v>
       </c>
@@ -10626,7 +10605,7 @@
         <v>0.65029800000000004</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>2029</v>
       </c>
@@ -10642,7 +10621,7 @@
         <v>0.63135699999999995</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>2030</v>
       </c>
@@ -10658,7 +10637,7 @@
         <v>0.61296799999999996</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>2031</v>
       </c>
@@ -10674,7 +10653,7 @@
         <v>0.59511499999999995</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2032</v>
       </c>
@@ -10690,7 +10669,7 @@
         <v>0.57778099999999999</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>2033</v>
       </c>
@@ -10706,7 +10685,7 @@
         <v>0.56095300000000003</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>2034</v>
       </c>
@@ -10722,7 +10701,7 @@
         <v>0.54461400000000004</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>2035</v>
       </c>
@@ -10752,7 +10731,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:AI47"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -10760,17 +10739,17 @@
     <col min="33" max="35" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="57" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="57" t="s">
         <v>182</v>
       </c>
@@ -10877,7 +10856,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -10984,7 +10963,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -11091,7 +11070,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -11198,7 +11177,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>101</v>
       </c>
@@ -11305,7 +11284,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>123</v>
       </c>
@@ -11412,7 +11391,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>44</v>
       </c>
@@ -11519,7 +11498,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -11626,7 +11605,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>75</v>
       </c>
@@ -11733,7 +11712,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>83</v>
       </c>
@@ -11840,7 +11819,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -11947,7 +11926,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>79</v>
       </c>
@@ -12054,7 +12033,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>113</v>
       </c>
@@ -12161,7 +12140,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>115</v>
       </c>
@@ -12268,7 +12247,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>97</v>
       </c>
@@ -12375,7 +12354,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>111</v>
       </c>
@@ -12482,7 +12461,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>127</v>
       </c>
@@ -12589,7 +12568,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -12696,7 +12675,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>99</v>
       </c>
@@ -12803,7 +12782,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>131</v>
       </c>
@@ -12910,7 +12889,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>129</v>
       </c>
@@ -13017,7 +12996,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A27" s="57" t="s">
         <v>234</v>
       </c>
@@ -13124,7 +13103,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>47</v>
       </c>
@@ -13231,7 +13210,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>50</v>
       </c>
@@ -13338,7 +13317,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>52</v>
       </c>
@@ -13445,7 +13424,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>101</v>
       </c>
@@ -13552,7 +13531,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>123</v>
       </c>
@@ -13659,7 +13638,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>44</v>
       </c>
@@ -13766,7 +13745,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>73</v>
       </c>
@@ -13873,7 +13852,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>75</v>
       </c>
@@ -13980,7 +13959,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>83</v>
       </c>
@@ -14087,7 +14066,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>77</v>
       </c>
@@ -14194,7 +14173,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>79</v>
       </c>
@@ -14301,7 +14280,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>113</v>
       </c>
@@ -14408,7 +14387,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>115</v>
       </c>
@@ -14515,7 +14494,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>97</v>
       </c>
@@ -14622,7 +14601,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>111</v>
       </c>
@@ -14729,7 +14708,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>127</v>
       </c>
@@ -14836,7 +14815,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>63</v>
       </c>
@@ -14943,7 +14922,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>99</v>
       </c>
@@ -15050,7 +15029,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>131</v>
       </c>
@@ -15157,7 +15136,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>129</v>
       </c>
@@ -15272,18 +15251,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AL776"/>
-  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="51.86328125" style="21" customWidth="1"/>
-    <col min="2" max="2" width="12.73046875" style="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.265625" style="21" customWidth="1"/>
-    <col min="4" max="4" width="9.59765625" style="21" customWidth="1"/>
-    <col min="5" max="38" width="7.59765625" style="21" customWidth="1"/>
-    <col min="39" max="39" width="12.59765625" style="21" customWidth="1"/>
-    <col min="40" max="16384" width="12.59765625" style="21"/>
+    <col min="1" max="1" width="51.85546875" style="21" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" style="21" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" style="21" customWidth="1"/>
+    <col min="5" max="38" width="7.5703125" style="21" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="21" customWidth="1"/>
+    <col min="40" max="16384" width="12.5703125" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>138</v>
       </c>
@@ -15325,7 +15304,7 @@
       <c r="AK1" s="20"/>
       <c r="AL1" s="20"/>
     </row>
-    <row r="2" spans="1:38" ht="92.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:38" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>139</v>
       </c>
@@ -15367,7 +15346,7 @@
       <c r="AK2" s="23"/>
       <c r="AL2" s="23"/>
     </row>
-    <row r="3" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
         <v>140</v>
       </c>
@@ -15409,7 +15388,7 @@
       <c r="AK3" s="23"/>
       <c r="AL3" s="23"/>
     </row>
-    <row r="4" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
         <v>141</v>
       </c>
@@ -15453,7 +15432,7 @@
       <c r="AK4" s="23"/>
       <c r="AL4" s="23"/>
     </row>
-    <row r="5" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
         <v>142</v>
       </c>
@@ -15497,7 +15476,7 @@
       <c r="AK5" s="23"/>
       <c r="AL5" s="23"/>
     </row>
-    <row r="6" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="56" t="s">
         <v>143</v>
       </c>
@@ -15559,7 +15538,7 @@
       <c r="AK6" s="23"/>
       <c r="AL6" s="23"/>
     </row>
-    <row r="7" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="21">
         <v>2023</v>
       </c>
@@ -15591,7 +15570,7 @@
         <v>2032</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="24" t="s">
         <v>144</v>
       </c>
@@ -15636,7 +15615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="24" t="s">
         <v>145</v>
       </c>
@@ -15681,7 +15660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
         <v>146</v>
       </c>
@@ -15726,7 +15705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>147</v>
       </c>
@@ -15768,7 +15747,7 @@
       <c r="AK12" s="20"/>
       <c r="AL12" s="20"/>
     </row>
-    <row r="13" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="24">
         <v>2022</v>
       </c>
@@ -15803,7 +15782,7 @@
         <v>2032</v>
       </c>
     </row>
-    <row r="14" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
         <v>148</v>
       </c>
@@ -15842,10 +15821,10 @@
         <v>0.57778099999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="24"/>
     </row>
-    <row r="16" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:38" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="24" t="s">
         <v>149</v>
       </c>
@@ -15853,22 +15832,22 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="17" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="24"/>
     </row>
-    <row r="18" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="19" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="24" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="20" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="24" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="21" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="22" spans="1:33" ht="39.4" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="1:33" ht="39.4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="24" t="s">
         <v>152</v>
       </c>
@@ -15882,7 +15861,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="23" spans="1:33" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:33" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="24" t="s">
         <v>156</v>
       </c>
@@ -15897,7 +15876,7 @@
         <v>5883.9075000000003</v>
       </c>
     </row>
-    <row r="24" spans="1:33" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:33" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="24" t="s">
         <v>159</v>
       </c>
@@ -15912,7 +15891,7 @@
         <v>5883.9075000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:33" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:33" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="24" t="s">
         <v>161</v>
       </c>
@@ -15927,13 +15906,13 @@
         <v>31380.84</v>
       </c>
     </row>
-    <row r="26" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="27" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="24" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="28" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="28" t="s">
         <v>164</v>
       </c>
@@ -15970,7 +15949,7 @@
       <c r="AF28" s="28"/>
       <c r="AG28" s="28"/>
     </row>
-    <row r="29" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="29" t="s">
         <v>165</v>
       </c>
@@ -16007,7 +15986,7 @@
       <c r="AF29" s="28"/>
       <c r="AG29" s="28"/>
     </row>
-    <row r="30" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="29" t="s">
         <v>166</v>
       </c>
@@ -16044,7 +16023,7 @@
       <c r="AF30" s="28"/>
       <c r="AG30" s="28"/>
     </row>
-    <row r="31" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="28" t="s">
         <v>167</v>
       </c>
@@ -16102,7 +16081,7 @@
       <c r="AE31" s="28"/>
       <c r="AF31" s="28"/>
     </row>
-    <row r="32" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:33" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="28" t="s">
         <v>168</v>
       </c>
@@ -16160,7 +16139,7 @@
       <c r="AE32" s="32"/>
       <c r="AF32" s="28"/>
     </row>
-    <row r="33" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="28" t="s">
         <v>169</v>
       </c>
@@ -16218,7 +16197,7 @@
       <c r="AE33" s="32"/>
       <c r="AF33" s="28"/>
     </row>
-    <row r="34" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="28" t="s">
         <v>170</v>
       </c>
@@ -16276,7 +16255,7 @@
       <c r="AE34" s="32"/>
       <c r="AF34" s="28"/>
     </row>
-    <row r="36" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="24" t="s">
         <v>171</v>
       </c>
@@ -16343,746 +16322,746 @@
       <c r="AC36" s="25"/>
       <c r="AD36" s="25"/>
     </row>
-    <row r="37" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="38" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="39" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="40" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="41" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="42" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="43" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="44" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="45" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="46" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="47" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="48" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="49" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="50" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="51" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="52" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="53" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="54" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="55" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="56" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="57" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="58" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="59" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="60" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="61" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="62" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="63" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="64" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="65" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="66" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="67" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="68" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="69" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="70" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="71" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="72" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="73" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="74" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="75" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="76" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="77" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="78" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="79" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="80" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="81" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="82" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="83" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="84" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="85" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="86" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="87" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="88" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="89" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="90" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="91" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="92" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="93" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="94" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="95" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="96" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="97" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="98" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="99" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="100" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="101" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="102" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="103" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="104" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="105" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="106" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="107" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="108" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="109" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="110" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="111" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="112" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="113" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="114" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="115" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="116" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="117" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="118" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="119" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="120" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="121" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="122" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="123" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="124" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="125" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="126" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="127" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="128" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="129" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="130" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="131" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="132" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="133" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="134" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="135" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="136" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="137" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="138" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="139" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="140" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="141" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="142" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="143" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="144" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="145" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="146" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="147" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="148" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="149" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="150" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="151" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="152" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="153" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="154" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="155" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="156" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="157" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="158" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="159" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="160" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="161" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="162" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="163" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="164" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="165" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="166" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="167" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="168" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="169" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="170" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="171" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="172" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="173" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="174" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="175" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="176" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="177" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="178" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="179" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="180" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="181" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="182" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="183" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="184" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="185" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="186" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="187" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="188" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="189" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="190" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="191" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="192" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="193" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="194" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="195" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="196" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="197" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="198" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="199" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="200" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="201" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="202" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="203" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="204" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="205" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="206" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="207" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="208" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="209" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="210" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="211" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="212" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="213" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="214" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="215" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="216" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="217" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="218" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="219" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="220" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="221" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="222" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="223" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="224" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="225" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="226" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="227" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="228" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="229" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="230" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="231" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="232" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="233" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="234" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="235" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="236" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="237" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="238" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="239" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="240" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="241" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="242" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="243" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="244" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="245" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="246" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="247" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="248" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="249" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="250" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="251" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="252" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="253" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="254" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="255" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="256" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="257" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="258" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="259" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="260" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="261" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="262" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="263" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="264" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="265" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="266" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="267" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="268" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="269" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="270" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="271" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="272" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="273" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="274" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="275" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="276" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="277" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="278" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="279" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="280" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="281" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="282" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="283" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="284" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="285" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="286" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="287" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="288" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="289" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="290" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="291" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="292" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="293" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="294" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="295" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="296" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="297" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="298" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="299" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="300" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="301" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="302" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="303" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="304" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="305" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="306" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="307" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="308" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="309" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="310" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="311" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="312" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="313" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="314" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="315" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="316" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="317" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="318" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="319" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="320" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="321" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="322" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="323" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="324" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="325" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="326" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="327" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="328" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="329" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="330" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="331" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="332" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="333" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="334" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="335" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="336" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="337" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="338" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="339" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="340" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="341" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="342" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="343" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="344" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="345" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="346" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="347" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="348" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="349" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="350" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="351" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="352" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="353" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="354" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="355" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="356" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="357" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="358" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="359" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="360" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="361" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="362" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="363" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="364" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="365" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="366" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="367" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="368" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="369" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="370" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="371" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="372" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="373" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="374" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="375" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="376" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="377" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="378" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="379" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="380" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="381" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="382" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="383" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="384" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="385" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="386" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="387" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="388" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="389" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="390" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="391" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="392" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="393" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="394" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="395" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="396" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="397" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="398" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="399" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="400" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="401" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="402" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="403" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="404" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="405" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="406" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="407" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="408" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="409" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="410" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="411" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="412" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="413" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="414" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="415" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="416" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="417" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="418" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="419" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="420" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="421" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="422" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="423" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="424" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="425" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="426" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="427" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="428" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="429" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="430" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="431" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="432" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="433" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="434" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="435" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="436" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="437" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="438" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="439" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="440" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="441" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="442" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="443" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="444" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="445" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="446" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="447" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="448" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="449" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="450" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="451" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="452" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="453" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="454" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="455" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="456" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="457" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="458" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="459" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="460" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="461" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="462" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="463" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="464" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="465" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="466" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="467" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="468" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="469" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="470" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="471" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="472" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="473" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="474" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="475" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="476" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="477" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="478" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="479" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="480" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="481" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="482" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="483" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="484" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="485" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="486" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="487" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="488" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="489" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="490" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="491" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="492" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="493" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="494" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="495" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="496" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="497" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="498" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="499" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="500" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="501" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="502" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="503" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="504" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="505" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="506" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="507" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="508" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="509" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="510" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="511" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="512" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="513" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="514" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="515" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="516" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="517" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="518" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="519" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="520" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="521" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="522" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="523" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="524" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="525" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="526" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="527" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="528" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="529" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="530" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="531" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="532" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="533" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="534" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="535" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="536" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="537" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="538" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="539" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="540" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="541" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="542" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="543" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="544" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="545" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="546" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="547" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="548" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="549" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="550" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="551" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="552" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="553" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="554" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="555" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="556" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="557" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="558" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="559" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="560" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="561" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="562" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="563" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="564" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="565" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="566" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="567" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="568" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="569" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="570" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="571" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="572" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="573" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="574" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="575" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="576" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="577" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="578" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="579" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="580" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="581" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="582" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="583" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="584" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="585" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="586" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="587" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="588" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="589" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="590" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="591" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="592" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="593" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="594" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="595" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="596" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="597" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="598" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="599" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="600" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="601" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="602" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="603" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="604" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="605" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="606" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="607" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="608" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="609" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="610" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="611" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="612" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="613" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="614" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="615" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="616" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="617" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="618" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="619" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="620" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="621" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="622" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="623" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="624" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="625" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="626" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="627" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="628" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="629" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="630" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="631" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="632" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="633" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="634" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="635" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="636" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="637" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="638" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="639" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="640" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="641" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="642" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="643" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="644" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="645" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="646" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="647" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="648" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="649" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="650" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="651" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="652" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="653" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="654" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="655" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="656" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="657" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="658" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="659" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="660" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="661" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="662" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="663" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="664" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="665" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="666" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="667" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="668" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="669" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="670" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="671" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="672" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="673" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="674" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="675" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="676" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="677" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="678" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="679" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="680" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="681" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="682" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="683" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="684" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="685" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="686" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="687" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="688" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="689" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="690" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="691" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="692" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="693" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="694" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="695" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="696" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="697" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="698" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="699" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="700" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="701" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="702" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="703" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="704" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="705" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="706" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="707" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="708" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="709" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="710" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="711" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="712" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="713" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="714" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="715" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="716" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="717" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="718" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="719" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="720" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="721" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="722" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="723" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="724" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="725" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="726" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="727" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="728" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="729" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="730" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="731" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="732" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="733" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="734" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="735" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="736" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="737" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="738" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="739" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="740" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="741" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="742" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="743" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="744" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="745" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="746" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="747" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="748" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="749" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="750" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="751" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="752" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="753" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="754" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="755" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="756" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="757" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="758" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="759" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="760" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="761" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="762" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="763" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="764" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="765" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="766" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="767" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="768" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="769" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="770" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="771" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="772" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="773" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="774" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="775" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="776" ht="13.15" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="37" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:32" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="49" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="50" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="51" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="52" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="53" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="54" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="55" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="57" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="58" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="59" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="60" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="61" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="62" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="63" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="64" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="65" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="66" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="67" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="68" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="69" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="70" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="71" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="72" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="73" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="74" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="76" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="77" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="78" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="80" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="81" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="82" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="83" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="85" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="86" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="87" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="89" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="90" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="91" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="92" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="94" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="96" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="97" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="98" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="99" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="100" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="101" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="102" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="103" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="104" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="105" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="106" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="107" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="108" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="109" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="110" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="111" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="112" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="113" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="114" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="115" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="116" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="117" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="118" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="119" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="120" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="121" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="122" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="123" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="124" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="125" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="126" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="127" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="128" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="129" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="130" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="131" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="132" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="133" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="134" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="135" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="136" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="137" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="138" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="139" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="140" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="141" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="142" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="143" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="144" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="145" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="146" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="147" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="148" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="149" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="150" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="151" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="152" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="153" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="154" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="155" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="156" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="157" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="158" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="159" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="160" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="161" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="162" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="163" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="164" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="165" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="166" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="167" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="168" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="169" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="170" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="171" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="172" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="173" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="174" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="175" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="176" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="177" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="178" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="179" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="180" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="181" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="182" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="183" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="184" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="185" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="186" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="187" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="188" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="189" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="190" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="191" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="192" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="193" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="194" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="195" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="196" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="197" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="198" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="199" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="200" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="201" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="202" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="203" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="204" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="205" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="206" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="207" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="208" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="209" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="210" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="211" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="212" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="213" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="214" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="215" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="216" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="217" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="218" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="219" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="220" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="221" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="222" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="223" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="224" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="225" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="226" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="227" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="228" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="229" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="230" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="231" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="232" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="233" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="234" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="235" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="236" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="237" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="238" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="239" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="240" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="241" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="242" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="243" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="244" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="245" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="246" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="247" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="248" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="249" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="250" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="251" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="252" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="253" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="254" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="255" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="256" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="257" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="258" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="259" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="260" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="261" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="262" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="263" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="264" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="265" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="266" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="267" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="268" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="269" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="270" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="271" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="272" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="273" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="274" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="275" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="276" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="277" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="278" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="279" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="280" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="281" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="282" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="283" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="284" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="285" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="286" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="287" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="288" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="289" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="290" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="291" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="292" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="293" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="294" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="295" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="296" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="297" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="298" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="299" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="300" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="301" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="302" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="303" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="304" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="305" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="306" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="307" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="308" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="309" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="310" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="311" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="312" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="313" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="314" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="315" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="316" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="317" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="318" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="319" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="320" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="321" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="322" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="323" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="324" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="325" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="326" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="327" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="328" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="329" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="330" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="331" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="332" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="333" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="334" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="335" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="336" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="337" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="338" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="339" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="340" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="341" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="342" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="343" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="344" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="345" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="346" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="347" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="348" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="349" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="350" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="351" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="352" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="353" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="354" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="355" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="356" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="357" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="358" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="359" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="360" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="361" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="362" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="363" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="364" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="365" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="366" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="367" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="368" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="369" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="370" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="371" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="372" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="373" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="374" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="375" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="376" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="377" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="378" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="379" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="380" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="381" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="382" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="383" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="384" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="385" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="386" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="387" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="388" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="389" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="390" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="391" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="392" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="393" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="394" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="395" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="396" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="397" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="398" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="399" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="400" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="401" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="402" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="403" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="404" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="405" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="406" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="407" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="408" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="409" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="410" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="411" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="412" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="413" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="414" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="415" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="416" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="417" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="418" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="419" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="420" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="421" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="422" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="423" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="424" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="425" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="426" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="427" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="428" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="429" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="430" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="431" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="432" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="433" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="434" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="435" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="436" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="437" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="438" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="439" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="440" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="441" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="442" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="443" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="444" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="445" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="446" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="447" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="448" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="449" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="450" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="451" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="452" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="453" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="454" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="455" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="456" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="457" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="458" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="459" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="460" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="461" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="462" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="463" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="464" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="465" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="466" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="467" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="468" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="469" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="470" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="471" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="472" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="473" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="474" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="475" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="476" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="477" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="478" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="479" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="480" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="481" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="482" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="483" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="484" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="485" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="486" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="487" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="488" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="489" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="490" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="491" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="492" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="493" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="494" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="495" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="496" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="497" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="498" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="499" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="500" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="501" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="502" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="503" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="504" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="505" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="506" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="507" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="508" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="509" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="510" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="511" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="512" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="513" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="514" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="515" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="516" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="517" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="518" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="519" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="520" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="521" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="522" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="523" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="524" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="525" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="526" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="527" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="528" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="529" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="530" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="531" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="532" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="533" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="534" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="535" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="536" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="537" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="538" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="539" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="540" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="541" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="542" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="543" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="544" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="545" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="546" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="547" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="548" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="549" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="550" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="551" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="552" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="553" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="554" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="555" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="556" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="557" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="558" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="559" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="560" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="561" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="562" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="563" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="564" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="565" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="566" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="567" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="568" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="569" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="570" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="571" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="572" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="573" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="574" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="575" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="576" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="577" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="578" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="579" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="580" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="581" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="582" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="583" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="584" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="585" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="586" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="587" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="588" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="589" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="590" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="591" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="592" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="593" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="594" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="595" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="596" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="597" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="598" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="599" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="600" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="601" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="602" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="603" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="604" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="605" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="606" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="607" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="608" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="609" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="610" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="611" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="612" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="613" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="614" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="615" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="616" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="617" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="618" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="619" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="620" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="621" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="622" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="623" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="624" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="625" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="626" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="627" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="628" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="629" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="630" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="631" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="632" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="633" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="634" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="635" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="636" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="637" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="638" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="639" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="640" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="641" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="642" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="643" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="644" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="645" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="646" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="647" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="648" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="649" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="650" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="651" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="652" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="653" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="654" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="655" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="656" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="657" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="658" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="659" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="660" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="661" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="662" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="663" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="664" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="665" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="666" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="667" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="668" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="669" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="670" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="671" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="672" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="673" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="674" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="675" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="676" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="677" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="678" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="679" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="680" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="681" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="682" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="683" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="684" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="685" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="686" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="687" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="688" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="689" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="690" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="691" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="692" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="693" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="694" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="695" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="696" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="697" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="698" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="699" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="700" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="701" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="702" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="703" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="704" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="705" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="706" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="707" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="708" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="709" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="710" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="711" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="712" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="713" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="714" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="715" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="716" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="717" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="718" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="719" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="720" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="721" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="722" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="723" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="724" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="725" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="726" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="727" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="728" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="729" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="730" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="731" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="732" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="733" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="734" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="735" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="736" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="737" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="738" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="739" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="740" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="741" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="742" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="743" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="744" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="745" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="746" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="747" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="748" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="749" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="750" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="751" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="752" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="753" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="754" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="755" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="756" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="757" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="758" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="759" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="760" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="761" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="762" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="763" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="764" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="765" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="766" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="767" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="768" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="769" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="770" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="771" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="772" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="773" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="774" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="775" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="776" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -17095,7 +17074,7 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17107,13 +17086,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
-    <col min="2" max="2" width="9.59765625" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -17208,7 +17187,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -17333,7 +17312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -17428,7 +17407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -17523,7 +17502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -17618,7 +17597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -17743,7 +17722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -17838,7 +17817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -17973,13 +17952,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
-    <col min="4" max="4" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -18074,7 +18053,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -18084,45 +18063,38 @@
       <c r="C2">
         <v>0</v>
       </c>
-      <c r="D2" s="54">
+      <c r="D2">
         <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!C14*'Commercial Vehicles'!$B16</f>
         <v>25920.503200000003</v>
       </c>
-      <c r="E2" s="54">
+      <c r="E2">
         <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!D14*'Commercial Vehicles'!$B16</f>
         <v>25177.910400000001</v>
       </c>
-      <c r="F2" s="54">
+      <c r="F2">
         <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!E14*'Commercial Vehicles'!$B16</f>
         <v>24444.571199999998</v>
       </c>
-      <c r="G2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!F14*'Commercial Vehicles'!$B16</f>
-        <v>23732.594400000002</v>
-      </c>
-      <c r="H2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!G14*'Commercial Vehicles'!$B16</f>
-        <v>23041.360800000002</v>
-      </c>
-      <c r="I2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!H14*'Commercial Vehicles'!$B16</f>
-        <v>22370.251200000002</v>
-      </c>
-      <c r="J2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!I14*'Commercial Vehicles'!$B16</f>
-        <v>21718.680799999998</v>
-      </c>
-      <c r="K2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!J14*'Commercial Vehicles'!$B16</f>
-        <v>21086.099199999997</v>
-      </c>
-      <c r="L2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!K14*'Commercial Vehicles'!$B16</f>
-        <v>20471.955999999998</v>
-      </c>
-      <c r="M2" s="54">
-        <f>'Commercial Vehicles'!$B4*'Commercial Vehicles'!L14*'Commercial Vehicles'!$B16</f>
-        <v>19875.666399999998</v>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -18179,7 +18151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -18274,7 +18246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -18369,7 +18341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -18464,7 +18436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -18475,7 +18447,7 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <f t="shared" ref="D6:M6" si="0">D2</f>
+        <f t="shared" ref="D6:F6" si="0">D2</f>
         <v>25920.503200000003</v>
       </c>
       <c r="E6">
@@ -18487,32 +18459,25 @@
         <v>24444.571199999998</v>
       </c>
       <c r="G6">
-        <f t="shared" si="0"/>
-        <v>23732.594400000002</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <f t="shared" si="0"/>
-        <v>23041.360800000002</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
-        <v>22370.251200000002</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <f t="shared" si="0"/>
-        <v>21718.680799999998</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <f t="shared" si="0"/>
-        <v>21086.099199999997</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <f t="shared" si="0"/>
-        <v>20471.955999999998</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <f t="shared" si="0"/>
-        <v>19875.666399999998</v>
+        <v>0</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -18569,7 +18534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -18664,7 +18629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -18675,7 +18640,7 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <f t="shared" ref="D8:M8" si="1">D2</f>
+        <f t="shared" ref="D8:F8" si="1">D2</f>
         <v>25920.503200000003</v>
       </c>
       <c r="E8">
@@ -18687,32 +18652,25 @@
         <v>24444.571199999998</v>
       </c>
       <c r="G8">
-        <f t="shared" si="1"/>
-        <v>23732.594400000002</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <f t="shared" si="1"/>
-        <v>23041.360800000002</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <f t="shared" si="1"/>
-        <v>22370.251200000002</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <f t="shared" si="1"/>
-        <v>21718.680799999998</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <f t="shared" si="1"/>
-        <v>21086.099199999997</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <f t="shared" si="1"/>
-        <v>20471.955999999998</v>
+        <v>0</v>
       </c>
       <c r="M8">
-        <f t="shared" si="1"/>
-        <v>19875.666399999998</v>
+        <v>0</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -18780,12 +18738,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -18880,7 +18838,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -18975,7 +18933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -19070,7 +19028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -19165,7 +19123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -19260,7 +19218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -19355,7 +19313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -19450,7 +19408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>
@@ -19556,12 +19514,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1328125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>172</v>
       </c>
@@ -19656,7 +19614,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>173</v>
       </c>
@@ -19751,7 +19709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>174</v>
       </c>
@@ -19846,7 +19804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -19941,7 +19899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>176</v>
       </c>
@@ -20036,7 +19994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>177</v>
       </c>
@@ -20131,7 +20089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>178</v>
       </c>
@@ -20226,7 +20184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>179</v>
       </c>

</xml_diff>